<commit_message>
Reformulação da lista de requisito
</commit_message>
<xml_diff>
--- a/DocumentçãoEngenharia/ListaRequisitoEstacionamento.xlsx
+++ b/DocumentçãoEngenharia/ListaRequisitoEstacionamento.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29917"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFC2437C-9CB5-4193-810F-6510154D4C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A78198E1-AB1F-4F85-8317-093BF6513239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,8 +52,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -118,7 +126,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>